<commit_message>
added trim resistor to BoM, added Vref trim invention to spec
</commit_message>
<xml_diff>
--- a/docs/DAC3_Prototype_BOM.xlsx
+++ b/docs/DAC3_Prototype_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/waynesankey/Documents/audio/dac3/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFDF3CB5-B307-CD49-B421-855D49C8F780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B23561E-CE60-3741-8C64-7D2EC1818F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11080" yWindow="1860" windowWidth="39620" windowHeight="29040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="197">
   <si>
     <t>DAC3 Prototype — Bill of Materials</t>
   </si>
@@ -614,6 +614,21 @@
   </si>
   <si>
     <t>2R ladder rungs made from 2x series R - better for layout, other reasons.</t>
+  </si>
+  <si>
+    <t>Ladder Trim</t>
+  </si>
+  <si>
+    <t>C25077</t>
+  </si>
+  <si>
+    <t>R 10 ohms 1%</t>
+  </si>
+  <si>
+    <t>R 10 ohms 1%, 0402 -55℃~+155℃ 10Ω 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>Use on 8 msbs to get most of the benefit</t>
   </si>
 </sst>
 </file>
@@ -3455,23 +3470,40 @@
         <v>191</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="42" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
+      <c r="B28" s="31" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>195</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>113</v>
+      </c>
       <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="G28" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="H28" s="13">
+        <f>8*4</f>
+        <v>32</v>
+      </c>
+      <c r="I28" s="15">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="J28" s="15">
+        <f t="shared" si="1"/>
+        <v>0.224</v>
       </c>
       <c r="K28" s="14"/>
       <c r="L28" s="16"/>
-      <c r="M28" s="14"/>
+      <c r="M28" s="31" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
@@ -3893,11 +3925,11 @@
       </c>
       <c r="H53" s="20">
         <f>SUM(H5:H51)</f>
-        <v>644</v>
+        <v>676</v>
       </c>
       <c r="J53" s="21">
         <f>SUM(J5:J51)</f>
-        <v>412.78679999999997</v>
+        <v>413.01079999999996</v>
       </c>
     </row>
   </sheetData>
@@ -4478,19 +4510,19 @@
     <row r="54" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A54" s="23">
         <f>COUNTA(Prototype!C5:C51)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B54" s="23">
         <f>SUM(Prototype!H5:H51)</f>
-        <v>644</v>
+        <v>676</v>
       </c>
       <c r="C54" s="24">
         <f>SUM(Prototype!J5:J51)</f>
-        <v>412.78679999999997</v>
+        <v>413.01079999999996</v>
       </c>
       <c r="D54" s="24">
         <f>IFERROR(SUM(Prototype!J5:J51)/SUM(Prototype!H5:H51),0)</f>
-        <v>0.64097329192546582</v>
+        <v>0.6109627218934911</v>
       </c>
       <c r="E54" s="23">
         <f>SUMPRODUCT(((Prototype!E5:E51&lt;&gt;"")/COUNTIF(Prototype!E5:E51,Prototype!E5:E51&amp;"")))</f>

</xml_diff>